<commit_message>
Implement breakout child sub-interfaces and shuffle harnesses (D13)
Introduce `a_parent` and `b_parent` columns in cabling sheets to allow the creation of virtual child interfaces under specified physical parents. Update validation logic to enforce correct formatting and relationships between parents and children. Enhance documentation to reflect these changes, including operator runbook updates and examples for using the new columns. Adjust importer logic to handle the new interface creation process, ensuring backward compatibility with existing sheets. This implementation supports advanced cabling scenarios while maintaining the integrity of existing functionality.
</commit_message>
<xml_diff>
--- a/samples/3_cabling_breakout_invalid.xlsx
+++ b/samples/3_cabling_breakout_invalid.xlsx
@@ -417,23 +417,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,55 +458,75 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>a_parent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>a_interface_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>b_end</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>b_end_kind</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>b_port</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>b_port_side</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>b_parent</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>b_interface_type</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>cable_type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>cable_profile</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>cable_group</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>cable_status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>length</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>length_unit</t>
         </is>
@@ -521,60 +545,68 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>swp4</t>
+          <t>swp4s0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp4</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>F9</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
         <is>
           <t>mmf-om4</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>breakout-1c4p-4c1p</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>leaf01-swp4</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>brk-overflow</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>connected</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>BRK-0002</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -593,40 +625,48 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>swp4</t>
+          <t>swp4s1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>F10</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>leaf01-swp4</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>brk-overflow</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -641,40 +681,48 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>swp4</t>
+          <t>swp4s2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>F11</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>leaf01-swp4</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>brk-overflow</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -689,40 +737,48 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>swp4</t>
+          <t>swp4s3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>F12</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>leaf01-swp4</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>brk-overflow</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -737,40 +793,48 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>swp4</t>
+          <t>swp4s4</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp4</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>F13</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>leaf01-swp4</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>brk-overflow</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -785,60 +849,68 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>swp5</t>
+          <t>swp5s0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>F14</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>mmf-om4</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>breakout-1c2p-2c1p</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>leaf01-swp5</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>brk-conflict</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
         <is>
           <t>connected</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>BRK-0003</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -857,44 +929,52 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>swp5</t>
+          <t>swp5s1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp5</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>F15</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
         <is>
           <t>smf-os2</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>leaf01-swp5</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>brk-conflict</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -909,60 +989,68 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>swp6</t>
+          <t>swp6s0</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp6</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>F16</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
         <is>
           <t>mmf-om4</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>breakout-1c2p-2c1p</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>leaf01-swp6-a</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>brk-duplicate-a</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>connected</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>BRK-0004</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -981,60 +1069,68 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>swp6</t>
+          <t>swp6s1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>lab1-dh1-r01-leaf01:swp6</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>lab1-dh1-r01-pp02</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>panel</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>F17</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>front</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
         <is>
           <t>mmf-om4</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>breakout-1c2p-2c1p</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>leaf01-swp6-b</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>brk-duplicate-b</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
         <is>
           <t>connected</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>BRK-0005</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>m</t>
         </is>

</xml_diff>

<commit_message>
Enhance environment configuration and documentation for NetBox integration
Update `.env.example` to include optional `NETBOX_REVERT_TOKEN` for improved security and flexibility in API interactions. Introduce `REVERT_PLAN_EXPIRY_MINUTES` to manage the time frame for successful revert confirmations. Add a new Excel template for cabling imports to facilitate advanced configurations. Revise README and design documentation to reflect these changes, ensuring users are informed about the new environment variables and their implications for deployment.
</commit_message>
<xml_diff>
--- a/samples/3_cabling_breakout_invalid.xlsx
+++ b/samples/3_cabling_breakout_invalid.xlsx
@@ -423,7 +423,7 @@
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -550,7 +550,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp4</t>
+          <t>swp4</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp4</t>
+          <t>swp4</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -686,7 +686,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp4</t>
+          <t>swp4</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp4</t>
+          <t>swp4</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -798,7 +798,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp4</t>
+          <t>swp4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -854,7 +854,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp5</t>
+          <t>swp5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -934,7 +934,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp5</t>
+          <t>swp5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -994,7 +994,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp6</t>
+          <t>swp6</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>lab1-dh1-r01-leaf01:swp6</t>
+          <t>swp6</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>

</xml_diff>